<commit_message>
Update preparation documents per CEO decisions
Keeps the hero headline as decided, separates example fees from
confirmed values in the profit calculator and adds a step-by-step example,
adds a 10-product shortlist with verified and unverified data marked, and
an iPhone guide for unpublishing the old GitHub Pages demo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UUBHitTXQWV1Q7wYtqUhDv
</commit_message>
<xml_diff>
--- a/vorbereitung/gewinnrechner.xlsx
+++ b/vorbereitung/gewinnrechner.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Anleitung" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Annahmen" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Gewinnrechner" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Beispielrechnung" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -68,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="101">
   <si>
     <t xml:space="preserve">Gewinnrechner – Anleitung</t>
   </si>
@@ -85,6 +86,12 @@
     <t xml:space="preserve">4. Spalte "Bewertung": Verlust (rot), knapp = unter 15 % Marge (orange), ok (grün).</t>
   </si>
   <si>
+    <t xml:space="preserve">5. Blatt "Beispielrechnung": zeigt Schritt für Schritt, wie Einkauf, Versand, Gebühren, Retourenreserve und Gewinn zusammenhängen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Spalte "Status" im Blatt "Annahmen": BESTÄTIGT / UNBESTÄTIGT / BEISPIEL / EINGABE.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Farben: blaue Schrift auf Gelb = Eingabe · schwarz = Formel · grün = Wert aus dem Blatt "Annahmen".</t>
   </si>
   <si>
@@ -106,6 +113,9 @@
     <t xml:space="preserve">Wert</t>
   </si>
   <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hinweis / Quelle</t>
   </si>
   <si>
@@ -115,55 +125,67 @@
     <t xml:space="preserve">Nein</t>
   </si>
   <si>
-    <t xml:space="preserve">Bei "Ja" wird keine Umsatzsteuer abgezogen (Annahme: Kleinunternehmerregelung). Mit Steuerberater klären.</t>
+    <t xml:space="preserve">EINGABE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deine Entscheidung (mit Steuerberater klären). Bei "Ja" wird keine Umsatzsteuer abgezogen.</t>
   </si>
   <si>
     <t xml:space="preserve">Umsatzsteuersatz</t>
   </si>
   <si>
-    <t xml:space="preserve">Regelsatz Deutschland 19 %. Ob für einzelne Produkte ein anderer Satz gilt, mit Steuerberater klären.</t>
+    <t xml:space="preserve">BESTÄTIGT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesetzlicher Regelsatz Deutschland 19 % (§ 12 Abs. 1 UStG). Ob für einzelne Produkte etwas anderes gilt: Steuerberater.</t>
   </si>
   <si>
     <t xml:space="preserve">Zahlungsgebühr in % vom Bruttobetrag</t>
   </si>
   <si>
-    <t xml:space="preserve">BEISPIELWERT. Echte Gebühr beim gewählten Zahlungsanbieter / Shopify-Tarif prüfen.</t>
+    <t xml:space="preserve">BEISPIEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platzhalter. Echte Gebühr beim gewählten Zahlungsanbieter / Shopify-Tarif ablesen.</t>
   </si>
   <si>
     <t xml:space="preserve">Zahlungsgebühr fix pro Bestellung (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">BEISPIELWERT. Beim Zahlungsanbieter prüfen.</t>
+    <t xml:space="preserve">Platzhalter. Beim Zahlungsanbieter ablesen.</t>
   </si>
   <si>
     <t xml:space="preserve">Shopify-Monatsgebühr (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Laut Vergleichsportal (qualimero.com, 2026) Basic ca. 33 € netto/Monat bei monatlicher Zahlung. Auf shopify.com/de prüfen.</t>
+    <t xml:space="preserve">UNBESTÄTIGT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drittquelle qualimero.com/blog/shopify-preise (2026): Basic ca. 33 € netto/Monat bei monatlicher Zahlung. Nicht auf shopify.com geprüft.</t>
   </si>
   <si>
     <t xml:space="preserve">Weitere feste Monatskosten (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">BEISPIELWERT, z. B. Apps, Rechtstexte-Abo, Domain anteilig.</t>
+    <t xml:space="preserve">Platzhalter, z. B. Apps, Rechtstexte-Abo, Domain anteilig.</t>
   </si>
   <si>
     <t xml:space="preserve">Erwartete Bestellungen pro Monat</t>
   </si>
   <si>
-    <t xml:space="preserve">BEISPIELWERT. Verteilt die festen Kosten auf jede Bestellung.</t>
+    <t xml:space="preserve">Platzhalter. Verteilt die festen Kosten auf jede Bestellung.</t>
   </si>
   <si>
     <t xml:space="preserve">Retourenquote</t>
   </si>
   <si>
-    <t xml:space="preserve">BEISPIELWERT. Anteil der Bestellungen, die zurückkommen.</t>
+    <t xml:space="preserve">Platzhalter. Anteil der Bestellungen, die zurückkommen.</t>
   </si>
   <si>
     <t xml:space="preserve">Kosten pro Retoure (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">BEISPIELWERT, z. B. Rücksendeetikett, nicht wiederverkaufbare Ware anteilig.</t>
+    <t xml:space="preserve">Platzhalter, z. B. Rücksendeetikett, nicht wiederverkaufbare Ware anteilig.</t>
   </si>
   <si>
     <t xml:space="preserve">Feste Kosten pro Bestellung (€)</t>
@@ -178,6 +200,9 @@
     <t xml:space="preserve">Berechnet: Retourenquote × Kosten pro Retoure</t>
   </si>
   <si>
+    <t xml:space="preserve">Status-Legende: BESTÄTIGT = gesetzlich bzw. belegt · UNBESTÄTIGT = aus Drittquelle, nicht beim Anbieter geprüft · BEISPIEL = erfundener Platzhalter · EINGABE = deine Entscheidung</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gewinnrechner pro Produkt (eine Bestellung = ein Stück)</t>
   </si>
   <si>
@@ -239,6 +264,114 @@
   </si>
   <si>
     <t xml:space="preserve">z. B. Printful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beispielrechnung: wie der Gewinn pro Bestellung entsteht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEISPIELZAHLEN – kein geprüftes Angebot. Gelbe Felder ändern, der Rest rechnet mit den Werten aus dem Blatt "Annahmen".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eingabe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hinweis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEISPIEL Hunde-Fleecejacke (Print on Demand)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name frei wählbar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verkaufspreis an Kunden, brutto (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEISPIEL – dein Shop-Preis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Versandkosten, die der Kunde zahlt, brutto (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEISPIEL – 0, wenn du Versand nicht berechnest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einkaufspreis Ware beim Anbieter (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEISPIEL – echter Wert aus dem Anbieter-Konto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Versand vom Anbieter zum Kunden (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechenschritt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betrag (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">So entsteht die Zahl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kunde zahlt insgesamt (brutto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verkaufspreis + Versand vom Kunden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Umsatzsteuer ans Finanzamt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 % sind im Bruttopreis enthalten (entfällt bei Kleinunternehmer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERGEBNIS: Umsatz netto (bleibt bei dir)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Einkauf Ware</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preis beim Anbieter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Versand Anbieter → Kunde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zahlst du an den Anbieter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Zahlungsgebühr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% vom Bruttobetrag + fixer Betrag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Plattform- und Fixkosten-Anteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopify + Apps etc. geteilt durch Bestellungen pro Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Retourenreserve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rücklage: Retourenquote × Kosten pro Retoure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Werbekosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERGEBNIS: Gewinn pro Bestellung (vor Einkommensteuer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nettoumsatz minus alle Kosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marge vom Nettoumsatz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faustregel im Rechner: unter 15 % = knapp</t>
   </si>
 </sst>
 </file>
@@ -330,7 +463,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -347,6 +480,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCFE2F3"/>
+        <bgColor rgb="FFD9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor rgb="FFCFE2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor rgb="FFFCE5CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE5CD"/>
+        <bgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -399,7 +556,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -424,12 +581,28 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -461,6 +634,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -521,7 +702,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFCFE2F3"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -739,7 +920,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="130"/>
@@ -771,21 +952,31 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
+      <c r="A7" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="A8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -804,156 +995,191 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="105"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B6" s="7" t="n">
         <v>0.19</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>17</v>
+      <c r="C6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B7" s="7" t="n">
         <v>0.029</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>19</v>
+      <c r="C7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B8" s="10" t="n">
         <v>0.25</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>21</v>
+      <c r="C8" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B9" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>23</v>
+      <c r="C9" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>25</v>
+      <c r="D10" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B11" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>27</v>
+      <c r="C11" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B12" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>29</v>
+      <c r="C12" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="B13" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>31</v>
+      <c r="C13" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="10" t="n">
+      <c r="A15" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="14" t="n">
         <f aca="false">IF(B11&gt;0,(B9+B10)/B11,0)</f>
         <v>1.76666666666667</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>33</v>
+      <c r="D15" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" s="10" t="n">
+      <c r="A16" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="14" t="n">
         <f aca="false">B12*B13</f>
         <v>0.6</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>35</v>
+      <c r="D16" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -994,195 +1220,195 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="I4" s="11" t="s">
+      <c r="A4" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="B4" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="11" t="s">
+      <c r="C4" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L4" s="11" t="s">
+      <c r="D4" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="E4" s="15" t="s">
         <v>50</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="M4" s="15" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="C5" s="10" t="n">
         <v>34.9</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="10" t="n">
         <v>18.5</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="16" t="n">
         <f aca="false">IF(C5="","",IF(Annahmen!$B$5="Ja",C5+D5,(C5+D5)/(1+Annahmen!$B$6)))</f>
         <v>29.327731092437</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="16" t="n">
         <f aca="false">IF(C5="","",(C5+D5)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>1.2621</v>
       </c>
-      <c r="I5" s="13" t="n">
+      <c r="I5" s="17" t="n">
         <f aca="false">IF(C5="","",Annahmen!$B$15)</f>
         <v>1.76666666666667</v>
       </c>
-      <c r="J5" s="13" t="n">
+      <c r="J5" s="17" t="n">
         <f aca="false">IF(C5="","",Annahmen!$B$16)</f>
         <v>0.6</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="K5" s="16" t="n">
         <f aca="false">IF(C5="","",G5-E5-F5-H5-I5-J5)</f>
         <v>3.19896442577031</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="L5" s="18" t="n">
         <f aca="false">IF(C5="","",IF(G5&gt;0,K5/G5,0))</f>
         <v>0.109076437440306</v>
       </c>
-      <c r="M5" s="15" t="str">
+      <c r="M5" s="19" t="str">
         <f aca="false">IF(C5="","",IF(K5&lt;0,"Verlust",IF(L5&lt;0.15,"knapp","ok")))</f>
         <v>knapp</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="C6" s="10" t="n">
         <v>29.9</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="10" t="n">
         <v>4.9</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="16" t="n">
         <f aca="false">IF(C6="","",IF(Annahmen!$B$5="Ja",C6+D6,(C6+D6)/(1+Annahmen!$B$6)))</f>
         <v>29.2436974789916</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="16" t="n">
         <f aca="false">IF(C6="","",(C6+D6)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>1.2592</v>
       </c>
-      <c r="I6" s="13" t="n">
+      <c r="I6" s="17" t="n">
         <f aca="false">IF(C6="","",Annahmen!$B$15)</f>
         <v>1.76666666666667</v>
       </c>
-      <c r="J6" s="13" t="n">
+      <c r="J6" s="17" t="n">
         <f aca="false">IF(C6="","",Annahmen!$B$16)</f>
         <v>0.6</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="K6" s="16" t="n">
         <f aca="false">IF(C6="","",G6-E6-F6-H6-I6-J6)</f>
         <v>8.61783081232493</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="L6" s="18" t="n">
         <f aca="false">IF(C6="","",IF(G6&gt;0,K6/G6,0))</f>
         <v>0.294690191570881</v>
       </c>
-      <c r="M6" s="15" t="str">
+      <c r="M6" s="19" t="str">
         <f aca="false">IF(C6="","",IF(K6&lt;0,"Verlust",IF(L6&lt;0.15,"knapp","ok")))</f>
         <v>ok</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" s="7" t="n">
+        <v>64</v>
+      </c>
+      <c r="C7" s="10" t="n">
         <v>19.9</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="16" t="n">
         <f aca="false">IF(C7="","",IF(Annahmen!$B$5="Ja",C7+D7,(C7+D7)/(1+Annahmen!$B$6)))</f>
         <v>16.7226890756303</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="16" t="n">
         <f aca="false">IF(C7="","",(C7+D7)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>0.8271</v>
       </c>
-      <c r="I7" s="13" t="n">
+      <c r="I7" s="17" t="n">
         <f aca="false">IF(C7="","",Annahmen!$B$15)</f>
         <v>1.76666666666667</v>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J7" s="17" t="n">
         <f aca="false">IF(C7="","",Annahmen!$B$16)</f>
         <v>0.6</v>
       </c>
-      <c r="K7" s="12" t="n">
+      <c r="K7" s="16" t="n">
         <f aca="false">IF(C7="","",G7-E7-F7-H7-I7-J7)</f>
         <v>-0.471077591036414</v>
       </c>
-      <c r="L7" s="14" t="n">
+      <c r="L7" s="18" t="n">
         <f aca="false">IF(C7="","",IF(G7&gt;0,K7/G7,0))</f>
         <v>-0.0281699664991624</v>
       </c>
-      <c r="M7" s="15" t="str">
+      <c r="M7" s="19" t="str">
         <f aca="false">IF(C7="","",IF(K7&lt;0,"Verlust",IF(L7&lt;0.15,"knapp","ok")))</f>
         <v>Verlust</v>
       </c>
@@ -1190,35 +1416,35 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="12" t="str">
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="16" t="str">
         <f aca="false">IF(C8="","",IF(Annahmen!$B$5="Ja",C8+D8,(C8+D8)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H8" s="12" t="str">
+      <c r="H8" s="16" t="str">
         <f aca="false">IF(C8="","",(C8+D8)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I8" s="13" t="str">
+      <c r="I8" s="17" t="str">
         <f aca="false">IF(C8="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J8" s="13" t="str">
+      <c r="J8" s="17" t="str">
         <f aca="false">IF(C8="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K8" s="12" t="str">
+      <c r="K8" s="16" t="str">
         <f aca="false">IF(C8="","",G8-E8-F8-H8-I8-J8)</f>
         <v/>
       </c>
-      <c r="L8" s="14" t="str">
+      <c r="L8" s="18" t="str">
         <f aca="false">IF(C8="","",IF(G8&gt;0,K8/G8,0))</f>
         <v/>
       </c>
-      <c r="M8" s="15" t="str">
+      <c r="M8" s="19" t="str">
         <f aca="false">IF(C8="","",IF(K8&lt;0,"Verlust",IF(L8&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1226,35 +1452,35 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="12" t="str">
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="16" t="str">
         <f aca="false">IF(C9="","",IF(Annahmen!$B$5="Ja",C9+D9,(C9+D9)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H9" s="12" t="str">
+      <c r="H9" s="16" t="str">
         <f aca="false">IF(C9="","",(C9+D9)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I9" s="13" t="str">
+      <c r="I9" s="17" t="str">
         <f aca="false">IF(C9="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J9" s="13" t="str">
+      <c r="J9" s="17" t="str">
         <f aca="false">IF(C9="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K9" s="12" t="str">
+      <c r="K9" s="16" t="str">
         <f aca="false">IF(C9="","",G9-E9-F9-H9-I9-J9)</f>
         <v/>
       </c>
-      <c r="L9" s="14" t="str">
+      <c r="L9" s="18" t="str">
         <f aca="false">IF(C9="","",IF(G9&gt;0,K9/G9,0))</f>
         <v/>
       </c>
-      <c r="M9" s="15" t="str">
+      <c r="M9" s="19" t="str">
         <f aca="false">IF(C9="","",IF(K9&lt;0,"Verlust",IF(L9&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1262,35 +1488,35 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="12" t="str">
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="16" t="str">
         <f aca="false">IF(C10="","",IF(Annahmen!$B$5="Ja",C10+D10,(C10+D10)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H10" s="12" t="str">
+      <c r="H10" s="16" t="str">
         <f aca="false">IF(C10="","",(C10+D10)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I10" s="13" t="str">
+      <c r="I10" s="17" t="str">
         <f aca="false">IF(C10="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J10" s="13" t="str">
+      <c r="J10" s="17" t="str">
         <f aca="false">IF(C10="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K10" s="12" t="str">
+      <c r="K10" s="16" t="str">
         <f aca="false">IF(C10="","",G10-E10-F10-H10-I10-J10)</f>
         <v/>
       </c>
-      <c r="L10" s="14" t="str">
+      <c r="L10" s="18" t="str">
         <f aca="false">IF(C10="","",IF(G10&gt;0,K10/G10,0))</f>
         <v/>
       </c>
-      <c r="M10" s="15" t="str">
+      <c r="M10" s="19" t="str">
         <f aca="false">IF(C10="","",IF(K10&lt;0,"Verlust",IF(L10&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1298,35 +1524,35 @@
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="12" t="str">
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="16" t="str">
         <f aca="false">IF(C11="","",IF(Annahmen!$B$5="Ja",C11+D11,(C11+D11)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H11" s="12" t="str">
+      <c r="H11" s="16" t="str">
         <f aca="false">IF(C11="","",(C11+D11)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I11" s="13" t="str">
+      <c r="I11" s="17" t="str">
         <f aca="false">IF(C11="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J11" s="13" t="str">
+      <c r="J11" s="17" t="str">
         <f aca="false">IF(C11="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K11" s="12" t="str">
+      <c r="K11" s="16" t="str">
         <f aca="false">IF(C11="","",G11-E11-F11-H11-I11-J11)</f>
         <v/>
       </c>
-      <c r="L11" s="14" t="str">
+      <c r="L11" s="18" t="str">
         <f aca="false">IF(C11="","",IF(G11&gt;0,K11/G11,0))</f>
         <v/>
       </c>
-      <c r="M11" s="15" t="str">
+      <c r="M11" s="19" t="str">
         <f aca="false">IF(C11="","",IF(K11&lt;0,"Verlust",IF(L11&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1334,35 +1560,35 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="12" t="str">
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="16" t="str">
         <f aca="false">IF(C12="","",IF(Annahmen!$B$5="Ja",C12+D12,(C12+D12)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H12" s="12" t="str">
+      <c r="H12" s="16" t="str">
         <f aca="false">IF(C12="","",(C12+D12)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I12" s="13" t="str">
+      <c r="I12" s="17" t="str">
         <f aca="false">IF(C12="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J12" s="13" t="str">
+      <c r="J12" s="17" t="str">
         <f aca="false">IF(C12="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K12" s="12" t="str">
+      <c r="K12" s="16" t="str">
         <f aca="false">IF(C12="","",G12-E12-F12-H12-I12-J12)</f>
         <v/>
       </c>
-      <c r="L12" s="14" t="str">
+      <c r="L12" s="18" t="str">
         <f aca="false">IF(C12="","",IF(G12&gt;0,K12/G12,0))</f>
         <v/>
       </c>
-      <c r="M12" s="15" t="str">
+      <c r="M12" s="19" t="str">
         <f aca="false">IF(C12="","",IF(K12&lt;0,"Verlust",IF(L12&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1370,35 +1596,35 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="12" t="str">
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="16" t="str">
         <f aca="false">IF(C13="","",IF(Annahmen!$B$5="Ja",C13+D13,(C13+D13)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H13" s="12" t="str">
+      <c r="H13" s="16" t="str">
         <f aca="false">IF(C13="","",(C13+D13)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I13" s="13" t="str">
+      <c r="I13" s="17" t="str">
         <f aca="false">IF(C13="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J13" s="13" t="str">
+      <c r="J13" s="17" t="str">
         <f aca="false">IF(C13="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K13" s="12" t="str">
+      <c r="K13" s="16" t="str">
         <f aca="false">IF(C13="","",G13-E13-F13-H13-I13-J13)</f>
         <v/>
       </c>
-      <c r="L13" s="14" t="str">
+      <c r="L13" s="18" t="str">
         <f aca="false">IF(C13="","",IF(G13&gt;0,K13/G13,0))</f>
         <v/>
       </c>
-      <c r="M13" s="15" t="str">
+      <c r="M13" s="19" t="str">
         <f aca="false">IF(C13="","",IF(K13&lt;0,"Verlust",IF(L13&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1406,35 +1632,35 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="12" t="str">
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="16" t="str">
         <f aca="false">IF(C14="","",IF(Annahmen!$B$5="Ja",C14+D14,(C14+D14)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H14" s="12" t="str">
+      <c r="H14" s="16" t="str">
         <f aca="false">IF(C14="","",(C14+D14)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I14" s="13" t="str">
+      <c r="I14" s="17" t="str">
         <f aca="false">IF(C14="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J14" s="13" t="str">
+      <c r="J14" s="17" t="str">
         <f aca="false">IF(C14="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K14" s="12" t="str">
+      <c r="K14" s="16" t="str">
         <f aca="false">IF(C14="","",G14-E14-F14-H14-I14-J14)</f>
         <v/>
       </c>
-      <c r="L14" s="14" t="str">
+      <c r="L14" s="18" t="str">
         <f aca="false">IF(C14="","",IF(G14&gt;0,K14/G14,0))</f>
         <v/>
       </c>
-      <c r="M14" s="15" t="str">
+      <c r="M14" s="19" t="str">
         <f aca="false">IF(C14="","",IF(K14&lt;0,"Verlust",IF(L14&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1442,35 +1668,35 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="12" t="str">
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="16" t="str">
         <f aca="false">IF(C15="","",IF(Annahmen!$B$5="Ja",C15+D15,(C15+D15)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H15" s="12" t="str">
+      <c r="H15" s="16" t="str">
         <f aca="false">IF(C15="","",(C15+D15)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I15" s="13" t="str">
+      <c r="I15" s="17" t="str">
         <f aca="false">IF(C15="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J15" s="13" t="str">
+      <c r="J15" s="17" t="str">
         <f aca="false">IF(C15="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K15" s="12" t="str">
+      <c r="K15" s="16" t="str">
         <f aca="false">IF(C15="","",G15-E15-F15-H15-I15-J15)</f>
         <v/>
       </c>
-      <c r="L15" s="14" t="str">
+      <c r="L15" s="18" t="str">
         <f aca="false">IF(C15="","",IF(G15&gt;0,K15/G15,0))</f>
         <v/>
       </c>
-      <c r="M15" s="15" t="str">
+      <c r="M15" s="19" t="str">
         <f aca="false">IF(C15="","",IF(K15&lt;0,"Verlust",IF(L15&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1478,35 +1704,35 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="12" t="str">
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="16" t="str">
         <f aca="false">IF(C16="","",IF(Annahmen!$B$5="Ja",C16+D16,(C16+D16)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H16" s="12" t="str">
+      <c r="H16" s="16" t="str">
         <f aca="false">IF(C16="","",(C16+D16)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I16" s="13" t="str">
+      <c r="I16" s="17" t="str">
         <f aca="false">IF(C16="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J16" s="13" t="str">
+      <c r="J16" s="17" t="str">
         <f aca="false">IF(C16="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K16" s="12" t="str">
+      <c r="K16" s="16" t="str">
         <f aca="false">IF(C16="","",G16-E16-F16-H16-I16-J16)</f>
         <v/>
       </c>
-      <c r="L16" s="14" t="str">
+      <c r="L16" s="18" t="str">
         <f aca="false">IF(C16="","",IF(G16&gt;0,K16/G16,0))</f>
         <v/>
       </c>
-      <c r="M16" s="15" t="str">
+      <c r="M16" s="19" t="str">
         <f aca="false">IF(C16="","",IF(K16&lt;0,"Verlust",IF(L16&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1514,35 +1740,35 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="12" t="str">
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="16" t="str">
         <f aca="false">IF(C17="","",IF(Annahmen!$B$5="Ja",C17+D17,(C17+D17)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H17" s="12" t="str">
+      <c r="H17" s="16" t="str">
         <f aca="false">IF(C17="","",(C17+D17)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I17" s="13" t="str">
+      <c r="I17" s="17" t="str">
         <f aca="false">IF(C17="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J17" s="13" t="str">
+      <c r="J17" s="17" t="str">
         <f aca="false">IF(C17="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K17" s="12" t="str">
+      <c r="K17" s="16" t="str">
         <f aca="false">IF(C17="","",G17-E17-F17-H17-I17-J17)</f>
         <v/>
       </c>
-      <c r="L17" s="14" t="str">
+      <c r="L17" s="18" t="str">
         <f aca="false">IF(C17="","",IF(G17&gt;0,K17/G17,0))</f>
         <v/>
       </c>
-      <c r="M17" s="15" t="str">
+      <c r="M17" s="19" t="str">
         <f aca="false">IF(C17="","",IF(K17&lt;0,"Verlust",IF(L17&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1550,35 +1776,35 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="12" t="str">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="16" t="str">
         <f aca="false">IF(C18="","",IF(Annahmen!$B$5="Ja",C18+D18,(C18+D18)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H18" s="12" t="str">
+      <c r="H18" s="16" t="str">
         <f aca="false">IF(C18="","",(C18+D18)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I18" s="13" t="str">
+      <c r="I18" s="17" t="str">
         <f aca="false">IF(C18="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J18" s="13" t="str">
+      <c r="J18" s="17" t="str">
         <f aca="false">IF(C18="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K18" s="12" t="str">
+      <c r="K18" s="16" t="str">
         <f aca="false">IF(C18="","",G18-E18-F18-H18-I18-J18)</f>
         <v/>
       </c>
-      <c r="L18" s="14" t="str">
+      <c r="L18" s="18" t="str">
         <f aca="false">IF(C18="","",IF(G18&gt;0,K18/G18,0))</f>
         <v/>
       </c>
-      <c r="M18" s="15" t="str">
+      <c r="M18" s="19" t="str">
         <f aca="false">IF(C18="","",IF(K18&lt;0,"Verlust",IF(L18&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1586,35 +1812,35 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="12" t="str">
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="16" t="str">
         <f aca="false">IF(C19="","",IF(Annahmen!$B$5="Ja",C19+D19,(C19+D19)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H19" s="12" t="str">
+      <c r="H19" s="16" t="str">
         <f aca="false">IF(C19="","",(C19+D19)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I19" s="13" t="str">
+      <c r="I19" s="17" t="str">
         <f aca="false">IF(C19="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J19" s="13" t="str">
+      <c r="J19" s="17" t="str">
         <f aca="false">IF(C19="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K19" s="12" t="str">
+      <c r="K19" s="16" t="str">
         <f aca="false">IF(C19="","",G19-E19-F19-H19-I19-J19)</f>
         <v/>
       </c>
-      <c r="L19" s="14" t="str">
+      <c r="L19" s="18" t="str">
         <f aca="false">IF(C19="","",IF(G19&gt;0,K19/G19,0))</f>
         <v/>
       </c>
-      <c r="M19" s="15" t="str">
+      <c r="M19" s="19" t="str">
         <f aca="false">IF(C19="","",IF(K19&lt;0,"Verlust",IF(L19&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1622,35 +1848,35 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="12" t="str">
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="16" t="str">
         <f aca="false">IF(C20="","",IF(Annahmen!$B$5="Ja",C20+D20,(C20+D20)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H20" s="12" t="str">
+      <c r="H20" s="16" t="str">
         <f aca="false">IF(C20="","",(C20+D20)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I20" s="13" t="str">
+      <c r="I20" s="17" t="str">
         <f aca="false">IF(C20="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J20" s="13" t="str">
+      <c r="J20" s="17" t="str">
         <f aca="false">IF(C20="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K20" s="12" t="str">
+      <c r="K20" s="16" t="str">
         <f aca="false">IF(C20="","",G20-E20-F20-H20-I20-J20)</f>
         <v/>
       </c>
-      <c r="L20" s="14" t="str">
+      <c r="L20" s="18" t="str">
         <f aca="false">IF(C20="","",IF(G20&gt;0,K20/G20,0))</f>
         <v/>
       </c>
-      <c r="M20" s="15" t="str">
+      <c r="M20" s="19" t="str">
         <f aca="false">IF(C20="","",IF(K20&lt;0,"Verlust",IF(L20&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1658,35 +1884,35 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="12" t="str">
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="16" t="str">
         <f aca="false">IF(C21="","",IF(Annahmen!$B$5="Ja",C21+D21,(C21+D21)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H21" s="12" t="str">
+      <c r="H21" s="16" t="str">
         <f aca="false">IF(C21="","",(C21+D21)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I21" s="13" t="str">
+      <c r="I21" s="17" t="str">
         <f aca="false">IF(C21="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J21" s="13" t="str">
+      <c r="J21" s="17" t="str">
         <f aca="false">IF(C21="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K21" s="12" t="str">
+      <c r="K21" s="16" t="str">
         <f aca="false">IF(C21="","",G21-E21-F21-H21-I21-J21)</f>
         <v/>
       </c>
-      <c r="L21" s="14" t="str">
+      <c r="L21" s="18" t="str">
         <f aca="false">IF(C21="","",IF(G21&gt;0,K21/G21,0))</f>
         <v/>
       </c>
-      <c r="M21" s="15" t="str">
+      <c r="M21" s="19" t="str">
         <f aca="false">IF(C21="","",IF(K21&lt;0,"Verlust",IF(L21&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1694,35 +1920,35 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="12" t="str">
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="16" t="str">
         <f aca="false">IF(C22="","",IF(Annahmen!$B$5="Ja",C22+D22,(C22+D22)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H22" s="12" t="str">
+      <c r="H22" s="16" t="str">
         <f aca="false">IF(C22="","",(C22+D22)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I22" s="13" t="str">
+      <c r="I22" s="17" t="str">
         <f aca="false">IF(C22="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J22" s="13" t="str">
+      <c r="J22" s="17" t="str">
         <f aca="false">IF(C22="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K22" s="12" t="str">
+      <c r="K22" s="16" t="str">
         <f aca="false">IF(C22="","",G22-E22-F22-H22-I22-J22)</f>
         <v/>
       </c>
-      <c r="L22" s="14" t="str">
+      <c r="L22" s="18" t="str">
         <f aca="false">IF(C22="","",IF(G22&gt;0,K22/G22,0))</f>
         <v/>
       </c>
-      <c r="M22" s="15" t="str">
+      <c r="M22" s="19" t="str">
         <f aca="false">IF(C22="","",IF(K22&lt;0,"Verlust",IF(L22&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1730,35 +1956,35 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="12" t="str">
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="16" t="str">
         <f aca="false">IF(C23="","",IF(Annahmen!$B$5="Ja",C23+D23,(C23+D23)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H23" s="12" t="str">
+      <c r="H23" s="16" t="str">
         <f aca="false">IF(C23="","",(C23+D23)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I23" s="13" t="str">
+      <c r="I23" s="17" t="str">
         <f aca="false">IF(C23="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J23" s="13" t="str">
+      <c r="J23" s="17" t="str">
         <f aca="false">IF(C23="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K23" s="12" t="str">
+      <c r="K23" s="16" t="str">
         <f aca="false">IF(C23="","",G23-E23-F23-H23-I23-J23)</f>
         <v/>
       </c>
-      <c r="L23" s="14" t="str">
+      <c r="L23" s="18" t="str">
         <f aca="false">IF(C23="","",IF(G23&gt;0,K23/G23,0))</f>
         <v/>
       </c>
-      <c r="M23" s="15" t="str">
+      <c r="M23" s="19" t="str">
         <f aca="false">IF(C23="","",IF(K23&lt;0,"Verlust",IF(L23&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1766,35 +1992,35 @@
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="12" t="str">
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="16" t="str">
         <f aca="false">IF(C24="","",IF(Annahmen!$B$5="Ja",C24+D24,(C24+D24)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H24" s="12" t="str">
+      <c r="H24" s="16" t="str">
         <f aca="false">IF(C24="","",(C24+D24)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I24" s="13" t="str">
+      <c r="I24" s="17" t="str">
         <f aca="false">IF(C24="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J24" s="13" t="str">
+      <c r="J24" s="17" t="str">
         <f aca="false">IF(C24="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K24" s="12" t="str">
+      <c r="K24" s="16" t="str">
         <f aca="false">IF(C24="","",G24-E24-F24-H24-I24-J24)</f>
         <v/>
       </c>
-      <c r="L24" s="14" t="str">
+      <c r="L24" s="18" t="str">
         <f aca="false">IF(C24="","",IF(G24&gt;0,K24/G24,0))</f>
         <v/>
       </c>
-      <c r="M24" s="15" t="str">
+      <c r="M24" s="19" t="str">
         <f aca="false">IF(C24="","",IF(K24&lt;0,"Verlust",IF(L24&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1802,35 +2028,35 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="12" t="str">
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="16" t="str">
         <f aca="false">IF(C25="","",IF(Annahmen!$B$5="Ja",C25+D25,(C25+D25)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H25" s="12" t="str">
+      <c r="H25" s="16" t="str">
         <f aca="false">IF(C25="","",(C25+D25)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I25" s="13" t="str">
+      <c r="I25" s="17" t="str">
         <f aca="false">IF(C25="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J25" s="13" t="str">
+      <c r="J25" s="17" t="str">
         <f aca="false">IF(C25="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K25" s="12" t="str">
+      <c r="K25" s="16" t="str">
         <f aca="false">IF(C25="","",G25-E25-F25-H25-I25-J25)</f>
         <v/>
       </c>
-      <c r="L25" s="14" t="str">
+      <c r="L25" s="18" t="str">
         <f aca="false">IF(C25="","",IF(G25&gt;0,K25/G25,0))</f>
         <v/>
       </c>
-      <c r="M25" s="15" t="str">
+      <c r="M25" s="19" t="str">
         <f aca="false">IF(C25="","",IF(K25&lt;0,"Verlust",IF(L25&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1838,35 +2064,35 @@
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="12" t="str">
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="16" t="str">
         <f aca="false">IF(C26="","",IF(Annahmen!$B$5="Ja",C26+D26,(C26+D26)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H26" s="12" t="str">
+      <c r="H26" s="16" t="str">
         <f aca="false">IF(C26="","",(C26+D26)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I26" s="13" t="str">
+      <c r="I26" s="17" t="str">
         <f aca="false">IF(C26="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J26" s="13" t="str">
+      <c r="J26" s="17" t="str">
         <f aca="false">IF(C26="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K26" s="12" t="str">
+      <c r="K26" s="16" t="str">
         <f aca="false">IF(C26="","",G26-E26-F26-H26-I26-J26)</f>
         <v/>
       </c>
-      <c r="L26" s="14" t="str">
+      <c r="L26" s="18" t="str">
         <f aca="false">IF(C26="","",IF(G26&gt;0,K26/G26,0))</f>
         <v/>
       </c>
-      <c r="M26" s="15" t="str">
+      <c r="M26" s="19" t="str">
         <f aca="false">IF(C26="","",IF(K26&lt;0,"Verlust",IF(L26&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1874,35 +2100,35 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="12" t="str">
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="16" t="str">
         <f aca="false">IF(C27="","",IF(Annahmen!$B$5="Ja",C27+D27,(C27+D27)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H27" s="12" t="str">
+      <c r="H27" s="16" t="str">
         <f aca="false">IF(C27="","",(C27+D27)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I27" s="13" t="str">
+      <c r="I27" s="17" t="str">
         <f aca="false">IF(C27="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J27" s="13" t="str">
+      <c r="J27" s="17" t="str">
         <f aca="false">IF(C27="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K27" s="12" t="str">
+      <c r="K27" s="16" t="str">
         <f aca="false">IF(C27="","",G27-E27-F27-H27-I27-J27)</f>
         <v/>
       </c>
-      <c r="L27" s="14" t="str">
+      <c r="L27" s="18" t="str">
         <f aca="false">IF(C27="","",IF(G27&gt;0,K27/G27,0))</f>
         <v/>
       </c>
-      <c r="M27" s="15" t="str">
+      <c r="M27" s="19" t="str">
         <f aca="false">IF(C27="","",IF(K27&lt;0,"Verlust",IF(L27&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1910,35 +2136,35 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="12" t="str">
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="16" t="str">
         <f aca="false">IF(C28="","",IF(Annahmen!$B$5="Ja",C28+D28,(C28+D28)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H28" s="12" t="str">
+      <c r="H28" s="16" t="str">
         <f aca="false">IF(C28="","",(C28+D28)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I28" s="13" t="str">
+      <c r="I28" s="17" t="str">
         <f aca="false">IF(C28="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J28" s="13" t="str">
+      <c r="J28" s="17" t="str">
         <f aca="false">IF(C28="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K28" s="12" t="str">
+      <c r="K28" s="16" t="str">
         <f aca="false">IF(C28="","",G28-E28-F28-H28-I28-J28)</f>
         <v/>
       </c>
-      <c r="L28" s="14" t="str">
+      <c r="L28" s="18" t="str">
         <f aca="false">IF(C28="","",IF(G28&gt;0,K28/G28,0))</f>
         <v/>
       </c>
-      <c r="M28" s="15" t="str">
+      <c r="M28" s="19" t="str">
         <f aca="false">IF(C28="","",IF(K28&lt;0,"Verlust",IF(L28&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1946,35 +2172,35 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="12" t="str">
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="16" t="str">
         <f aca="false">IF(C29="","",IF(Annahmen!$B$5="Ja",C29+D29,(C29+D29)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H29" s="12" t="str">
+      <c r="H29" s="16" t="str">
         <f aca="false">IF(C29="","",(C29+D29)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I29" s="13" t="str">
+      <c r="I29" s="17" t="str">
         <f aca="false">IF(C29="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J29" s="13" t="str">
+      <c r="J29" s="17" t="str">
         <f aca="false">IF(C29="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K29" s="12" t="str">
+      <c r="K29" s="16" t="str">
         <f aca="false">IF(C29="","",G29-E29-F29-H29-I29-J29)</f>
         <v/>
       </c>
-      <c r="L29" s="14" t="str">
+      <c r="L29" s="18" t="str">
         <f aca="false">IF(C29="","",IF(G29&gt;0,K29/G29,0))</f>
         <v/>
       </c>
-      <c r="M29" s="15" t="str">
+      <c r="M29" s="19" t="str">
         <f aca="false">IF(C29="","",IF(K29&lt;0,"Verlust",IF(L29&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -1982,35 +2208,35 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5"/>
       <c r="B30" s="5"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="12" t="str">
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="16" t="str">
         <f aca="false">IF(C30="","",IF(Annahmen!$B$5="Ja",C30+D30,(C30+D30)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H30" s="12" t="str">
+      <c r="H30" s="16" t="str">
         <f aca="false">IF(C30="","",(C30+D30)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I30" s="13" t="str">
+      <c r="I30" s="17" t="str">
         <f aca="false">IF(C30="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J30" s="13" t="str">
+      <c r="J30" s="17" t="str">
         <f aca="false">IF(C30="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K30" s="12" t="str">
+      <c r="K30" s="16" t="str">
         <f aca="false">IF(C30="","",G30-E30-F30-H30-I30-J30)</f>
         <v/>
       </c>
-      <c r="L30" s="14" t="str">
+      <c r="L30" s="18" t="str">
         <f aca="false">IF(C30="","",IF(G30&gt;0,K30/G30,0))</f>
         <v/>
       </c>
-      <c r="M30" s="15" t="str">
+      <c r="M30" s="19" t="str">
         <f aca="false">IF(C30="","",IF(K30&lt;0,"Verlust",IF(L30&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -2018,35 +2244,35 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="12" t="str">
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="16" t="str">
         <f aca="false">IF(C31="","",IF(Annahmen!$B$5="Ja",C31+D31,(C31+D31)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H31" s="12" t="str">
+      <c r="H31" s="16" t="str">
         <f aca="false">IF(C31="","",(C31+D31)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I31" s="13" t="str">
+      <c r="I31" s="17" t="str">
         <f aca="false">IF(C31="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J31" s="13" t="str">
+      <c r="J31" s="17" t="str">
         <f aca="false">IF(C31="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K31" s="12" t="str">
+      <c r="K31" s="16" t="str">
         <f aca="false">IF(C31="","",G31-E31-F31-H31-I31-J31)</f>
         <v/>
       </c>
-      <c r="L31" s="14" t="str">
+      <c r="L31" s="18" t="str">
         <f aca="false">IF(C31="","",IF(G31&gt;0,K31/G31,0))</f>
         <v/>
       </c>
-      <c r="M31" s="15" t="str">
+      <c r="M31" s="19" t="str">
         <f aca="false">IF(C31="","",IF(K31&lt;0,"Verlust",IF(L31&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -2054,35 +2280,35 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5"/>
       <c r="B32" s="5"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="12" t="str">
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="16" t="str">
         <f aca="false">IF(C32="","",IF(Annahmen!$B$5="Ja",C32+D32,(C32+D32)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H32" s="12" t="str">
+      <c r="H32" s="16" t="str">
         <f aca="false">IF(C32="","",(C32+D32)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I32" s="13" t="str">
+      <c r="I32" s="17" t="str">
         <f aca="false">IF(C32="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J32" s="13" t="str">
+      <c r="J32" s="17" t="str">
         <f aca="false">IF(C32="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K32" s="12" t="str">
+      <c r="K32" s="16" t="str">
         <f aca="false">IF(C32="","",G32-E32-F32-H32-I32-J32)</f>
         <v/>
       </c>
-      <c r="L32" s="14" t="str">
+      <c r="L32" s="18" t="str">
         <f aca="false">IF(C32="","",IF(G32&gt;0,K32/G32,0))</f>
         <v/>
       </c>
-      <c r="M32" s="15" t="str">
+      <c r="M32" s="19" t="str">
         <f aca="false">IF(C32="","",IF(K32&lt;0,"Verlust",IF(L32&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -2090,35 +2316,35 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="12" t="str">
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="16" t="str">
         <f aca="false">IF(C33="","",IF(Annahmen!$B$5="Ja",C33+D33,(C33+D33)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H33" s="12" t="str">
+      <c r="H33" s="16" t="str">
         <f aca="false">IF(C33="","",(C33+D33)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I33" s="13" t="str">
+      <c r="I33" s="17" t="str">
         <f aca="false">IF(C33="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J33" s="13" t="str">
+      <c r="J33" s="17" t="str">
         <f aca="false">IF(C33="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K33" s="12" t="str">
+      <c r="K33" s="16" t="str">
         <f aca="false">IF(C33="","",G33-E33-F33-H33-I33-J33)</f>
         <v/>
       </c>
-      <c r="L33" s="14" t="str">
+      <c r="L33" s="18" t="str">
         <f aca="false">IF(C33="","",IF(G33&gt;0,K33/G33,0))</f>
         <v/>
       </c>
-      <c r="M33" s="15" t="str">
+      <c r="M33" s="19" t="str">
         <f aca="false">IF(C33="","",IF(K33&lt;0,"Verlust",IF(L33&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -2126,35 +2352,35 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5"/>
       <c r="B34" s="5"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="12" t="str">
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="16" t="str">
         <f aca="false">IF(C34="","",IF(Annahmen!$B$5="Ja",C34+D34,(C34+D34)/(1+Annahmen!$B$6)))</f>
         <v/>
       </c>
-      <c r="H34" s="12" t="str">
+      <c r="H34" s="16" t="str">
         <f aca="false">IF(C34="","",(C34+D34)*Annahmen!$B$7+Annahmen!$B$8)</f>
         <v/>
       </c>
-      <c r="I34" s="13" t="str">
+      <c r="I34" s="17" t="str">
         <f aca="false">IF(C34="","",Annahmen!$B$15)</f>
         <v/>
       </c>
-      <c r="J34" s="13" t="str">
+      <c r="J34" s="17" t="str">
         <f aca="false">IF(C34="","",Annahmen!$B$16)</f>
         <v/>
       </c>
-      <c r="K34" s="12" t="str">
+      <c r="K34" s="16" t="str">
         <f aca="false">IF(C34="","",G34-E34-F34-H34-I34-J34)</f>
         <v/>
       </c>
-      <c r="L34" s="14" t="str">
+      <c r="L34" s="18" t="str">
         <f aca="false">IF(C34="","",IF(G34&gt;0,K34/G34,0))</f>
         <v/>
       </c>
-      <c r="M34" s="15" t="str">
+      <c r="M34" s="19" t="str">
         <f aca="false">IF(C34="","",IF(K34&lt;0,"Verlust",IF(L34&lt;0.15,"knapp","ok")))</f>
         <v/>
       </c>
@@ -2180,4 +2406,254 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="16" t="n">
+        <f aca="false">B6+B7</f>
+        <v>44.8</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <f aca="false">IF(Annahmen!$B$5="Ja",0,-(B13-B13/(1+Annahmen!$B$6)))</f>
+        <v>-7.15294117647058</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="20" t="n">
+        <f aca="false">B13+B14</f>
+        <v>37.6470588235294</v>
+      </c>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="16" t="n">
+        <f aca="false">-B8</f>
+        <v>-27</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" s="16" t="n">
+        <f aca="false">-B9</f>
+        <v>-5.5</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="16" t="n">
+        <f aca="false">-(B13*Annahmen!$B$7+Annahmen!$B$8)</f>
+        <v>-1.5492</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="16" t="n">
+        <f aca="false">-Annahmen!$B$15</f>
+        <v>-1.76666666666667</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" s="16" t="n">
+        <f aca="false">-Annahmen!$B$16</f>
+        <v>-0.6</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21" s="16" t="n">
+        <f aca="false">-B10</f>
+        <v>-3</v>
+      </c>
+      <c r="C21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B22" s="20" t="n">
+        <f aca="false">SUM(B15:B21)</f>
+        <v>-1.76880784313725</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B23" s="21" t="n">
+        <f aca="false">IF(B15&gt;0,B22/B15,0)</f>
+        <v>-0.0469839583333333</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>